<commit_message>
Ground-truth verification update via Scrapling for Comorin International School (https://cis.edu.in)
</commit_message>
<xml_diff>
--- a/kanyakumari_schools_verified_enriched_v2.xlsx
+++ b/kanyakumari_schools_verified_enriched_v2.xlsx
@@ -508,7 +508,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -19302,7 +19301,7 @@
       </c>
       <c r="C281" s="4" t="inlineStr">
         <is>
-          <t>COMERIN INTERNATIONAL ARALVOIMOZHY</t>
+          <t>Comorin International School</t>
         </is>
       </c>
       <c r="D281" s="5" t="inlineStr">
@@ -19332,27 +19331,27 @@
       </c>
       <c r="I281" s="4" t="inlineStr">
         <is>
-          <t>https://comerin.edu.in</t>
+          <t>https://cis.edu.in</t>
         </is>
       </c>
       <c r="J281" s="4" t="inlineStr">
         <is>
-          <t>Dr. K. George (Principal)</t>
+          <t>Er. E. Lekshmanan (Chairman) / Akash Elango Lekshmanan (Vice Chairman)</t>
         </is>
       </c>
       <c r="K281" s="4" t="inlineStr">
         <is>
-          <t>04652-263450</t>
+          <t>+91 94422 03041 / 04652-290933</t>
         </is>
       </c>
       <c r="L281" s="4" t="inlineStr">
         <is>
-          <t>info@comerin.edu.in</t>
+          <t>comorin@cis.edu.in / admin@cis.edu.in</t>
         </is>
       </c>
       <c r="M281" s="4" t="inlineStr">
         <is>
-          <t>Approx. 1,050</t>
+          <t>ICSE &amp; ISC (Class Pre-K to XII)</t>
         </is>
       </c>
       <c r="N281" s="7" t="inlineStr">
@@ -19362,7 +19361,7 @@
       </c>
       <c r="O281" s="4" t="inlineStr">
         <is>
-          <t>Comerin Educational Trust portal</t>
+          <t>Verified Ground Truth via Scrapling from https://cis.edu.in/ (Thiyagi Elango Memorial Trust; Chairman: Er. E. Lekshmanan; ICSE/ISC Affiliated; Admin: 04652-290933, Academics: 04652-290844)</t>
         </is>
       </c>
     </row>

</xml_diff>